<commit_message>
Add 12 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 77
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-15T02:16:22.807Z</t>
+    <t>2026-10-15T05:35:57.145Z</t>
   </si>
   <si>
     <t>Deutsch</t>
@@ -70,7 +70,7 @@
     <t>us/en</t>
   </si>
   <si>
-    <t>2026-10-15T02:36:42.677Z</t>
+    <t>2026-10-15T05:35:52.409Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -79,6 +79,27 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-profile","cards-profile"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:05:36.476Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
@@ -91,7 +112,7 @@
     <t>adventures-listing</t>
   </si>
   <si>
-    <t>2026-10-15T02:49:09.986Z</t>
+    <t>2026-10-15T04:05:16.444Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -100,6 +121,63 @@
     <t>https://wknd.site/us/en/adventures.html</t>
   </si>
   <si>
+    <t>us/en/ai-powered-search.report.json</t>
+  </si>
+  <si>
+    <t>["search"]</t>
+  </si>
+  <si>
+    <t>us/en/ai-powered-search</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:05:46.941Z</t>
+  </si>
+  <si>
+    <t>AI-Powered Search</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/ai-powered-search.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["hero","accordion"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faq-page</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:05:21.958Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns-featured","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:05:41.640Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
     <t>ca/en/adventures/yosemite-backpacking.report.json</t>
   </si>
   <si>
@@ -112,7 +190,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-10-15T02:33:57.665Z</t>
+    <t>2026-10-15T05:36:09.540Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -127,13 +205,49 @@
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>2026-10-15T02:49:55.303Z</t>
+    <t>2026-10-15T05:36:03.135Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>["hero","breadcrumbs","quote"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>magazine-article</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:08:43.016Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure</t>
+  </si>
+  <si>
+    <t>2026-10-15T04:08:48.481Z</t>
+  </si>
+  <si>
+    <t>Alaskan Adventure</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/members-only/alaskan-adventure.html</t>
   </si>
 </sst>
 </file>
@@ -522,11 +636,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="39" customWidth="1"/>
+    <col min="3" max="3" width="47" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
@@ -668,25 +782,181 @@
         <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" t="s">
+        <v>77</v>
+      </c>
+      <c r="H12" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>